<commit_message>
feat: actualizar propiedades en ColaboradorDTO, ajustar lógica en ColaboradorRepository y ColaboradorExtensions, y eliminar métodos obsoletos en AsistenciaService
</commit_message>
<xml_diff>
--- a/Campos API Colaboradores.xlsx
+++ b/Campos API Colaboradores.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tonovarela/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tonovarela/Documents/c#/apiBukLitoprocess/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EF8B77A5-F7DF-0142-BC54-4B75E78EA642}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42A98BCD-7F24-C844-B847-88FC1C50DDD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27720" yWindow="600" windowWidth="23480" windowHeight="26580" xr2:uid="{48F9F4EC-0B3B-42CC-A147-39E861EA5040}"/>
+    <workbookView xWindow="31560" yWindow="1420" windowWidth="23480" windowHeight="26560" xr2:uid="{48F9F4EC-0B3B-42CC-A147-39E861EA5040}"/>
   </bookViews>
   <sheets>
     <sheet name="Campos" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="158">
   <si>
     <t>Campo Intelisis</t>
   </si>
@@ -522,6 +522,9 @@
   </si>
   <si>
     <t>No hubo cambios</t>
+  </si>
+  <si>
+    <t>?????10-07-00-00</t>
   </si>
 </sst>
 </file>
@@ -1327,6 +1330,9 @@
       <c r="D11" s="9" t="s">
         <v>124</v>
       </c>
+      <c r="E11" t="s">
+        <v>11</v>
+      </c>
       <c r="F11" s="13" t="s">
         <v>139</v>
       </c>
@@ -1397,6 +1403,9 @@
       </c>
       <c r="D15" t="s">
         <v>32</v>
+      </c>
+      <c r="E15" t="s">
+        <v>11</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>33</v>
@@ -1417,7 +1426,9 @@
       <c r="D16" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="E16" s="4"/>
+      <c r="E16" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="F16" s="3" t="s">
         <v>33</v>
       </c>
@@ -1435,6 +1446,9 @@
       <c r="C17">
         <v>30</v>
       </c>
+      <c r="E17" t="s">
+        <v>11</v>
+      </c>
       <c r="F17" s="8" t="s">
         <v>37</v>
       </c>
@@ -1506,6 +1520,9 @@
       <c r="D21" s="9" t="s">
         <v>128</v>
       </c>
+      <c r="E21" t="s">
+        <v>11</v>
+      </c>
       <c r="F21" s="8" t="s">
         <v>37</v>
       </c>
@@ -1523,6 +1540,9 @@
       <c r="C22">
         <v>10</v>
       </c>
+      <c r="E22" t="s">
+        <v>11</v>
+      </c>
       <c r="F22" s="8" t="s">
         <v>37</v>
       </c>
@@ -1998,6 +2018,9 @@
       <c r="D45" s="9" t="s">
         <v>132</v>
       </c>
+      <c r="E45" t="s">
+        <v>11</v>
+      </c>
       <c r="F45" s="3" t="s">
         <v>33</v>
       </c>
@@ -2015,6 +2038,12 @@
       <c r="C46">
         <v>50</v>
       </c>
+      <c r="D46" t="s">
+        <v>157</v>
+      </c>
+      <c r="E46" t="s">
+        <v>11</v>
+      </c>
       <c r="F46" s="3" t="s">
         <v>33</v>
       </c>
@@ -2035,6 +2064,9 @@
       <c r="D47" t="s">
         <v>92</v>
       </c>
+      <c r="E47" t="s">
+        <v>11</v>
+      </c>
       <c r="F47" s="3" t="s">
         <v>33</v>
       </c>
@@ -2266,7 +2298,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="59" spans="1:7" ht="32" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>112</v>
       </c>

</xml_diff>

<commit_message>
Modulo de test implementado
</commit_message>
<xml_diff>
--- a/Campos API Colaboradores.xlsx
+++ b/Campos API Colaboradores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tonovarela/Documents/c#/apiBukLitoprocess/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4979EDC0-B9AE-0E4A-9197-AA451CB4288B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FCF3C4A-902E-B04B-8EA6-A80F7E37AFDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31560" yWindow="1420" windowWidth="23480" windowHeight="26560" xr2:uid="{48F9F4EC-0B3B-42CC-A147-39E861EA5040}"/>
+    <workbookView xWindow="27720" yWindow="600" windowWidth="23480" windowHeight="26560" xr2:uid="{48F9F4EC-0B3B-42CC-A147-39E861EA5040}"/>
   </bookViews>
   <sheets>
     <sheet name="Campos" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="159">
   <si>
     <t>Campo Intelisis</t>
   </si>
@@ -526,12 +526,15 @@
   <si>
     <t>?????10-07-00-00</t>
   </si>
+  <si>
+    <t>RESULTADO DE PRUEBAS</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -574,6 +577,13 @@
       <color rgb="FF7FDBCA"/>
       <name val="Monaco"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
@@ -632,7 +642,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -656,6 +666,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1148,6 +1159,9 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>158</v>
+      </c>
     </row>
     <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -1446,6 +1460,9 @@
       <c r="C17">
         <v>30</v>
       </c>
+      <c r="D17" t="s">
+        <v>38</v>
+      </c>
       <c r="E17" t="s">
         <v>11</v>
       </c>
@@ -1983,7 +2000,7 @@
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
+      <c r="A44" s="17" t="s">
         <v>87</v>
       </c>
       <c r="B44" t="s">
@@ -2029,7 +2046,7 @@
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
+      <c r="A46" s="17" t="s">
         <v>90</v>
       </c>
       <c r="B46" t="s">
@@ -2052,7 +2069,7 @@
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
+      <c r="A47" s="17" t="s">
         <v>91</v>
       </c>
       <c r="B47" t="s">

</xml_diff>